<commit_message>
docs: arrumando os valores do custo de implementação e as planilhas
</commit_message>
<xml_diff>
--- a/docs/public/sprints/sprint-3/1_Custo_POC.xlsx
+++ b/docs/public/sprints/sprint-3/1_Custo_POC.xlsx
@@ -118,13 +118,13 @@
     <t xml:space="preserve">Ambiente Red Hat/OpenShift</t>
   </si>
   <si>
-    <t xml:space="preserve">Equivalente pago ROSA — ver planilha 2</t>
+    <t xml:space="preserve">Cluster ROSA mínimo de não-produção — ver planilha 2</t>
   </si>
   <si>
     <t xml:space="preserve">Banco de dados Azure SQL</t>
   </si>
   <si>
-    <t xml:space="preserve">Equivalente pago — ver planilha 2</t>
+    <t xml:space="preserve">Compute serverless de desenvolvimento — ver planilha 2</t>
   </si>
   <si>
     <t xml:space="preserve">Docker e bibliotecas open source</t>
@@ -181,19 +181,19 @@
     <t xml:space="preserve">Hardware não suporta o OpenShift Local</t>
   </si>
   <si>
-    <t xml:space="preserve">Migração para ambiente gerenciado</t>
+    <t xml:space="preserve">Migração para cluster ROSA mínimo</t>
   </si>
   <si>
     <t xml:space="preserve">Volume ultrapassa a camada gratuita do Azure SQL</t>
   </si>
   <si>
-    <t xml:space="preserve">Reserva anual estimada</t>
+    <t xml:space="preserve">Compute serverless por 12 meses</t>
   </si>
   <si>
     <t xml:space="preserve">Necessidade de publicar o frontend durante a POC</t>
   </si>
   <si>
-    <t xml:space="preserve">Vercel Pro, 1 assento</t>
+    <t xml:space="preserve">Vercel Pro, 1 assento, 12 meses</t>
   </si>
   <si>
     <t xml:space="preserve">Pior caso quantificado</t>
@@ -894,7 +894,7 @@
         <v>31</v>
       </c>
       <c r="B25" s="15" t="n">
-        <v>6431.1</v>
+        <v>45503.73</v>
       </c>
       <c r="C25" s="15" t="n">
         <v>0</v>
@@ -908,7 +908,7 @@
         <v>33</v>
       </c>
       <c r="B26" s="15" t="n">
-        <v>1500</v>
+        <v>3060</v>
       </c>
       <c r="C26" s="15" t="n">
         <v>0</v>
@@ -965,7 +965,7 @@
       </c>
       <c r="B30" s="12" t="n">
         <f aca="false">SUM(B24:B29)</f>
-        <v>37331.1</v>
+        <v>77963.73</v>
       </c>
       <c r="C30" s="12" t="n">
         <f aca="false">SUM(C24:C29)</f>
@@ -1030,7 +1030,7 @@
         <v>52</v>
       </c>
       <c r="B42" s="15" t="n">
-        <v>6431.1</v>
+        <v>45503.73</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>53</v>
@@ -1041,7 +1041,7 @@
         <v>54</v>
       </c>
       <c r="B43" s="15" t="n">
-        <v>1500</v>
+        <v>3060</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>55</v>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="B45" s="12" t="n">
         <f aca="false">SUM(B42:B44)</f>
-        <v>9155.1</v>
+        <v>49787.73</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>